<commit_message>
09/10: reword regulatory framing (art. 13 scope, art. 50 duty split) and generalize ratio narration so printed metrics speak for themselves.
</commit_message>
<xml_diff>
--- a/09_ai-transparency-documentation/exercises/starter/model_card.xlsx
+++ b/09_ai-transparency-documentation/exercises/starter/model_card.xlsx
@@ -588,7 +588,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>REGULATORY CONTEXT: EU AI Act — FeedbackIQ-Sentiment-v3 is classified as Limited Risk in itself (no Annex III hit), but the deployment context with the EU customer triggers Article 13 transparency obligations and the customer's procurement process triggers Article 11 documentation review.</t>
+          <t>REGULATORY CONTEXT: EU AI Act — FeedbackIQ-Sentiment-v3 is classified as Limited Risk in itself (no Annex III hit); Article 13 transparency obligations attach only to high-risk systems, so the binding driver here is the EU customer's procurement process, which contractually requires Article 11-style technical documentation for vendor sign-off.</t>
         </is>
       </c>
     </row>
@@ -1288,12 +1288,12 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>Art. 50 — transparency obligation toward end users (deployer)</t>
+          <t>Art. 50 — transparency obligation toward end users (split provider / deployer duties)</t>
         </is>
       </c>
       <c r="C5" s="12" t="inlineStr">
         <is>
-          <t>[Your response here — what is NOT yet covered for Art. 50 deployer transparency? See the Article 11 Reference sheet for the Article 50 row.]</t>
+          <t>[Your response here — what is NOT yet covered for Art. 50 transparency (mind the provider/deployer duty split)? See the Article 11 Reference sheet for the Article 50 row.]</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -1662,7 +1662,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Disclosure obligations toward end users when they interact with AI systems — chatbot labels, deepfake labels, emotion recognition / biometric categorisation notice. Deployer obligation. Lives outside the Article 11 stack but cross-references it when end-user disclosure is needed.</t>
+          <t>Disclosure obligations toward end users when they interact with AI systems — provider duty for direct-interaction (chatbot) labels and synthetic-content marking (Art. 50(1)–(2)); deployer duty for emotion-recognition / biometric-categorisation notices and deepfake labelling (Art. 50(3)–(4)). Lives outside the Article 11 stack but cross-references it when end-user disclosure is needed.</t>
         </is>
       </c>
     </row>

</xml_diff>